<commit_message>
Improved handling of values as Currency and Percentages
</commit_message>
<xml_diff>
--- a/Templates/trading_journal_template.xlsx
+++ b/Templates/trading_journal_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/261a4915364edc4c/Coding/Projects/Trading Journal/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="721" documentId="11_F25DC773A252ABDACC10481179D95E825BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{123DD557-D6FE-460F-96DE-7547D1F3AA0C}"/>
+  <xr:revisionPtr revIDLastSave="722" documentId="11_F25DC773A252ABDACC10481179D95E825BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E6F7162-F4FB-4363-BE3C-2F199D288364}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Improvements" sheetId="13" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="384">
   <si>
     <t>Ideas</t>
   </si>
@@ -1195,6 +1195,12 @@
   </si>
   <si>
     <t>Trade Direction</t>
+  </si>
+  <si>
+    <t>Defines the maximum possible losses that could have taken place during the trade.</t>
+  </si>
+  <si>
+    <t>Defines the maximum possible profits that could have taken place during the trade.</t>
   </si>
 </sst>
 </file>
@@ -4296,7 +4302,7 @@
   <sheetPr codeName="Sheet10">
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="A4:F56"/>
+  <dimension ref="A4:F58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.7265625" customWidth="1"/>
@@ -4692,6 +4698,22 @@
       </c>
       <c r="F56" t="s">
         <v>107</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>144</v>
+      </c>
+      <c r="B57" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>145</v>
+      </c>
+      <c r="B58" t="s">
+        <v>383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>